<commit_message>
feat: add daily operations reports for 3rd and 4th September 2026, update continuous photo flow SOP guidelines
</commit_message>
<xml_diff>
--- a/Mucheru_World_of_Golf_Machinery_Cost_August_2026.xlsx
+++ b/Mucheru_World_of_Golf_Machinery_Cost_August_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\denni\Downloads\Reporting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A6B6E2-57EA-49E9-AC18-C3723CB253D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FC19AE-A3C9-4AB0-9687-B1606BEF6506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1793,16 +1793,43 @@
     <xf numFmtId="169" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
@@ -1815,46 +1842,17 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
@@ -1866,6 +1864,8 @@
     <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2198,7 +2198,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="112" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="106"/>
@@ -2221,7 +2221,7 @@
       <c r="S1" s="106"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="105" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="106"/>
@@ -2244,7 +2244,7 @@
       <c r="S2" s="106"/>
     </row>
     <row r="3" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="124" t="s">
+      <c r="A3" s="118" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="106"/>
@@ -2268,116 +2268,116 @@
     </row>
     <row r="4" spans="1:19" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="109" t="s">
+      <c r="A5" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="109" t="s">
+      <c r="B5" s="110"/>
+      <c r="C5" s="110"/>
+      <c r="D5" s="114" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="109" t="s">
+      <c r="E5" s="110"/>
+      <c r="F5" s="110"/>
+      <c r="G5" s="110"/>
+      <c r="H5" s="114" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="108"/>
-      <c r="L5" s="109" t="s">
+      <c r="I5" s="110"/>
+      <c r="J5" s="110"/>
+      <c r="K5" s="110"/>
+      <c r="L5" s="114" t="s">
         <v>6</v>
       </c>
-      <c r="M5" s="108"/>
-      <c r="N5" s="108"/>
-      <c r="O5" s="108"/>
-      <c r="P5" s="109" t="s">
+      <c r="M5" s="110"/>
+      <c r="N5" s="110"/>
+      <c r="O5" s="110"/>
+      <c r="P5" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="108"/>
-      <c r="R5" s="108"/>
-      <c r="S5" s="108"/>
+      <c r="Q5" s="110"/>
+      <c r="R5" s="110"/>
+      <c r="S5" s="110"/>
     </row>
     <row r="6" spans="1:19" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="122">
+      <c r="A6" s="115">
         <f>R41</f>
         <v>2790101.666666667</v>
       </c>
-      <c r="B6" s="108"/>
-      <c r="C6" s="108"/>
-      <c r="D6" s="117">
+      <c r="B6" s="110"/>
+      <c r="C6" s="110"/>
+      <c r="D6" s="109">
         <f>H41</f>
         <v>1046350</v>
       </c>
-      <c r="E6" s="108"/>
-      <c r="F6" s="108"/>
-      <c r="G6" s="108"/>
-      <c r="H6" s="117">
+      <c r="E6" s="110"/>
+      <c r="F6" s="110"/>
+      <c r="G6" s="110"/>
+      <c r="H6" s="109">
         <f>K41</f>
         <v>901751.66666666674</v>
       </c>
-      <c r="I6" s="108"/>
-      <c r="J6" s="108"/>
-      <c r="K6" s="108"/>
-      <c r="L6" s="107">
+      <c r="I6" s="110"/>
+      <c r="J6" s="110"/>
+      <c r="K6" s="110"/>
+      <c r="L6" s="125">
         <f>O41</f>
         <v>842000</v>
       </c>
-      <c r="M6" s="108"/>
-      <c r="N6" s="108"/>
-      <c r="O6" s="108"/>
-      <c r="P6" s="120" t="s">
+      <c r="M6" s="110"/>
+      <c r="N6" s="110"/>
+      <c r="O6" s="110"/>
+      <c r="P6" s="113" t="s">
         <v>8</v>
       </c>
-      <c r="Q6" s="108"/>
-      <c r="R6" s="108"/>
-      <c r="S6" s="108"/>
+      <c r="Q6" s="110"/>
+      <c r="R6" s="110"/>
+      <c r="S6" s="110"/>
     </row>
     <row r="7" spans="1:19" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="115" t="s">
+      <c r="A7" s="117" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="108"/>
-      <c r="C7" s="108"/>
-      <c r="D7" s="115" t="s">
+      <c r="B7" s="110"/>
+      <c r="C7" s="110"/>
+      <c r="D7" s="117" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="108"/>
-      <c r="F7" s="108"/>
-      <c r="G7" s="108"/>
-      <c r="H7" s="115" t="s">
+      <c r="E7" s="110"/>
+      <c r="F7" s="110"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="108"/>
-      <c r="J7" s="108"/>
-      <c r="K7" s="108"/>
-      <c r="L7" s="115" t="s">
+      <c r="I7" s="110"/>
+      <c r="J7" s="110"/>
+      <c r="K7" s="110"/>
+      <c r="L7" s="117" t="s">
         <v>12</v>
       </c>
-      <c r="M7" s="108"/>
-      <c r="N7" s="108"/>
-      <c r="O7" s="108"/>
-      <c r="P7" s="115" t="s">
+      <c r="M7" s="110"/>
+      <c r="N7" s="110"/>
+      <c r="O7" s="110"/>
+      <c r="P7" s="117" t="s">
         <v>13</v>
       </c>
-      <c r="Q7" s="108"/>
-      <c r="R7" s="108"/>
-      <c r="S7" s="108"/>
+      <c r="Q7" s="110"/>
+      <c r="R7" s="110"/>
+      <c r="S7" s="110"/>
     </row>
     <row r="8" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="121" t="s">
+      <c r="A8" s="107" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="106"/>
       <c r="C8" s="106"/>
       <c r="D8" s="106"/>
       <c r="E8" s="106"/>
-      <c r="F8" s="105" t="s">
+      <c r="F8" s="124" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="106"/>
       <c r="H8" s="106"/>
-      <c r="I8" s="113" t="s">
+      <c r="I8" s="122" t="s">
         <v>16</v>
       </c>
       <c r="J8" s="106"/>
@@ -2385,7 +2385,7 @@
       <c r="L8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="M8" s="114" t="s">
+      <c r="M8" s="123" t="s">
         <v>18</v>
       </c>
       <c r="N8" s="106"/>
@@ -2396,7 +2396,7 @@
       <c r="Q8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="R8" s="121" t="s">
+      <c r="R8" s="107" t="s">
         <v>21</v>
       </c>
       <c r="S8" s="106"/>
@@ -4431,13 +4431,13 @@
       </c>
     </row>
     <row r="41" spans="1:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="110" t="s">
+      <c r="A41" s="119" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="111"/>
-      <c r="C41" s="111"/>
-      <c r="D41" s="111"/>
-      <c r="E41" s="112"/>
+      <c r="B41" s="120"/>
+      <c r="C41" s="120"/>
+      <c r="D41" s="120"/>
+      <c r="E41" s="121"/>
       <c r="F41" s="71">
         <f>SUM(F10:F40)</f>
         <v>123.1</v>
@@ -4491,7 +4491,7 @@
       </c>
     </row>
     <row r="42" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="118" t="s">
+      <c r="A42" s="111" t="s">
         <v>159</v>
       </c>
       <c r="B42" s="106"/>
@@ -4535,7 +4535,7 @@
         <f>O41/15</f>
         <v>56133.333333333336</v>
       </c>
-      <c r="P42" s="123" t="s">
+      <c r="P42" s="116" t="s">
         <v>160</v>
       </c>
       <c r="Q42" s="106"/>
@@ -4548,14 +4548,14 @@
       </c>
     </row>
     <row r="43" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="118" t="s">
+      <c r="A43" s="111" t="s">
         <v>162</v>
       </c>
       <c r="B43" s="106"/>
       <c r="C43" s="106"/>
       <c r="D43" s="106"/>
       <c r="E43" s="106"/>
-      <c r="F43" s="116" t="s">
+      <c r="F43" s="108" t="s">
         <v>163</v>
       </c>
       <c r="G43" s="106"/>
@@ -4579,30 +4579,30 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A2:S2"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="F43:Q43"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="P6:S6"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="L5:O5"/>
-    <mergeCell ref="A43:E43"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="P42:Q42"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="P7:S7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A41:E41"/>
     <mergeCell ref="I8:K8"/>
     <mergeCell ref="M8:O8"/>
     <mergeCell ref="L7:O7"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="F43:Q43"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="L6:O6"/>
     <mergeCell ref="D5:G5"/>
     <mergeCell ref="H5:K5"/>
@@ -4630,7 +4630,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="112" t="s">
         <v>165</v>
       </c>
       <c r="B1" s="106"/>
@@ -4644,7 +4644,7 @@
       <c r="J1" s="106"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="105" t="s">
         <v>166</v>
       </c>
       <c r="B2" s="106"/>
@@ -4658,7 +4658,7 @@
       <c r="J2" s="106"/>
     </row>
     <row r="3" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="124" t="s">
+      <c r="A3" s="118" t="s">
         <v>167</v>
       </c>
       <c r="B3" s="106"/>
@@ -5103,18 +5103,18 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="73.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="112" t="s">
         <v>292</v>
       </c>
       <c r="B1" s="106"/>
@@ -5126,7 +5126,7 @@
       <c r="H1" s="106"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="105" t="s">
         <v>293</v>
       </c>
       <c r="B2" s="106"/>
@@ -5138,7 +5138,7 @@
       <c r="H2" s="106"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="124" t="s">
+      <c r="A3" s="118" t="s">
         <v>294</v>
       </c>
       <c r="B3" s="106"/>
@@ -5151,7 +5151,7 @@
     </row>
     <row r="4" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="135" t="s">
         <v>295</v>
       </c>
       <c r="B5" s="106"/>
@@ -5302,12 +5302,12 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="110" t="s">
+      <c r="A11" s="119" t="s">
         <v>324</v>
       </c>
-      <c r="B11" s="111"/>
-      <c r="C11" s="111"/>
-      <c r="D11" s="111"/>
+      <c r="B11" s="120"/>
+      <c r="C11" s="120"/>
+      <c r="D11" s="120"/>
       <c r="E11" s="79">
         <f>SUM(E7:E10)</f>
         <v>2790101.666666667</v>
@@ -5352,11 +5352,11 @@
       <c r="E14" s="102" t="s">
         <v>332</v>
       </c>
-      <c r="F14" s="135" t="s">
+      <c r="F14" s="133" t="s">
         <v>333</v>
       </c>
-      <c r="G14" s="136"/>
-      <c r="H14" s="136"/>
+      <c r="G14" s="134"/>
+      <c r="H14" s="134"/>
     </row>
     <row r="15" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="92" t="s">
@@ -5375,11 +5375,11 @@
         <f>D14/$D$18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F15" s="131" t="s">
+      <c r="F15" s="126" t="s">
         <v>337</v>
       </c>
-      <c r="G15" s="132"/>
-      <c r="H15" s="132"/>
+      <c r="G15" s="127"/>
+      <c r="H15" s="127"/>
     </row>
     <row r="16" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="88" t="s">
@@ -5398,11 +5398,11 @@
         <f>D15/$D$18</f>
         <v>14.986148711459146</v>
       </c>
-      <c r="F16" s="129" t="s">
+      <c r="F16" s="136" t="s">
         <v>341</v>
       </c>
-      <c r="G16" s="130"/>
-      <c r="H16" s="130"/>
+      <c r="G16" s="137"/>
+      <c r="H16" s="137"/>
     </row>
     <row r="17" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="92" t="s">
@@ -5421,11 +5421,11 @@
         <f>D16/$D$18</f>
         <v>5.6311589097604058</v>
       </c>
-      <c r="F17" s="131" t="s">
+      <c r="F17" s="126" t="s">
         <v>345</v>
       </c>
-      <c r="G17" s="132"/>
-      <c r="H17" s="132"/>
+      <c r="G17" s="127"/>
+      <c r="H17" s="127"/>
     </row>
     <row r="18" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="88" t="s">
@@ -5444,18 +5444,18 @@
         <f>D17/$D$18</f>
         <v>3.7238308919383329</v>
       </c>
-      <c r="F18" s="129" t="s">
+      <c r="F18" s="136" t="s">
         <v>349</v>
       </c>
-      <c r="G18" s="130"/>
-      <c r="H18" s="130"/>
+      <c r="G18" s="137"/>
+      <c r="H18" s="137"/>
     </row>
     <row r="19" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="133" t="s">
+      <c r="A19" s="131" t="s">
         <v>350</v>
       </c>
-      <c r="B19" s="127"/>
-      <c r="C19" s="127"/>
+      <c r="B19" s="129"/>
+      <c r="C19" s="129"/>
       <c r="D19" s="103">
         <f>SUM(D15:D18)</f>
         <v>2790101.67</v>
@@ -5467,12 +5467,12 @@
       <c r="F19" s="138" t="s">
         <v>351</v>
       </c>
-      <c r="G19" s="127"/>
-      <c r="H19" s="127"/>
+      <c r="G19" s="129"/>
+      <c r="H19" s="129"/>
     </row>
     <row r="20" spans="1:8" ht="14.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="134" t="s">
+      <c r="A21" s="132" t="s">
         <v>352</v>
       </c>
       <c r="B21" s="106"/>
@@ -5487,60 +5487,66 @@
       <c r="A22" s="128" t="s">
         <v>353</v>
       </c>
-      <c r="B22" s="127"/>
-      <c r="C22" s="126" t="s">
+      <c r="B22" s="129"/>
+      <c r="C22" s="130" t="s">
         <v>354</v>
       </c>
-      <c r="D22" s="127"/>
-      <c r="E22" s="127"/>
-      <c r="F22" s="127"/>
-      <c r="G22" s="127"/>
-      <c r="H22" s="127"/>
+      <c r="D22" s="129"/>
+      <c r="E22" s="129"/>
+      <c r="F22" s="129"/>
+      <c r="G22" s="129"/>
+      <c r="H22" s="129"/>
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="128" t="s">
         <v>355</v>
       </c>
-      <c r="B23" s="127"/>
-      <c r="C23" s="126" t="s">
+      <c r="B23" s="129"/>
+      <c r="C23" s="130" t="s">
         <v>356</v>
       </c>
-      <c r="D23" s="127"/>
-      <c r="E23" s="127"/>
-      <c r="F23" s="127"/>
-      <c r="G23" s="127"/>
-      <c r="H23" s="127"/>
+      <c r="D23" s="129"/>
+      <c r="E23" s="129"/>
+      <c r="F23" s="129"/>
+      <c r="G23" s="129"/>
+      <c r="H23" s="129"/>
     </row>
     <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="128" t="s">
         <v>357</v>
       </c>
-      <c r="B24" s="127"/>
-      <c r="C24" s="126" t="s">
+      <c r="B24" s="129"/>
+      <c r="C24" s="130" t="s">
         <v>358</v>
       </c>
-      <c r="D24" s="127"/>
-      <c r="E24" s="127"/>
-      <c r="F24" s="127"/>
-      <c r="G24" s="127"/>
-      <c r="H24" s="127"/>
+      <c r="D24" s="129"/>
+      <c r="E24" s="129"/>
+      <c r="F24" s="129"/>
+      <c r="G24" s="129"/>
+      <c r="H24" s="129"/>
     </row>
     <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="128" t="s">
         <v>359</v>
       </c>
-      <c r="B25" s="127"/>
-      <c r="C25" s="126" t="s">
+      <c r="B25" s="129"/>
+      <c r="C25" s="130" t="s">
         <v>360</v>
       </c>
-      <c r="D25" s="127"/>
-      <c r="E25" s="127"/>
-      <c r="F25" s="127"/>
-      <c r="G25" s="127"/>
-      <c r="H25" s="127"/>
+      <c r="D25" s="129"/>
+      <c r="E25" s="129"/>
+      <c r="F25" s="129"/>
+      <c r="G25" s="129"/>
+      <c r="H25" s="129"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="F17:H17"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A25:B25"/>
@@ -5557,12 +5563,6 @@
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="F19:H19"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="F17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>